<commit_message>
Added .gitignore, now have to remove the temp files, also added the final main model, some more collaborator data and comparisons, and another new analysis file, also some simulations of the main DHAM that worked
</commit_message>
<xml_diff>
--- a/data/Holdings/Museum_map.xlsx
+++ b/data/Holdings/Museum_map.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brinda/Documents/MRes project/data/Holdings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3978E550-C5CE-1647-AAC6-E582AF118B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A164480A-D911-5644-A9A0-701D9501C743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1580" yWindow="2000" windowWidth="26440" windowHeight="14280" xr2:uid="{C4C7C71C-19E0-2247-8E7D-B844CAD8A477}"/>
+    <workbookView xWindow="1580" yWindow="2000" windowWidth="26440" windowHeight="14280" activeTab="2" xr2:uid="{C4C7C71C-19E0-2247-8E7D-B844CAD8A477}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="League table" sheetId="2" r:id="rId2"/>
+    <sheet name="Field sites" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="82">
   <si>
     <t>Sr. No</t>
   </si>
@@ -227,9 +228,6 @@
     <t>NHMUK1</t>
   </si>
   <si>
-    <t>Difference</t>
-  </si>
-  <si>
     <t>NMK, Kenya</t>
   </si>
   <si>
@@ -240,6 +238,51 @@
   </si>
   <si>
     <t>PC</t>
+  </si>
+  <si>
+    <t>Field (IISER Tirupati)</t>
+  </si>
+  <si>
+    <t>University of Western Ontario</t>
+  </si>
+  <si>
+    <t>Field (Equatorial Guinea)</t>
+  </si>
+  <si>
+    <t>Field (Nigeria_Chima)</t>
+  </si>
+  <si>
+    <t>Field (Zambia_Chima)</t>
+  </si>
+  <si>
+    <t>Field (Thailand)</t>
+  </si>
+  <si>
+    <t>Field (Malaysia)</t>
+  </si>
+  <si>
+    <t>Field (Kenya)</t>
+  </si>
+  <si>
+    <t>Field (Equatorial Guinea_1.0)</t>
+  </si>
+  <si>
+    <t>Field (Ghana_1.0)</t>
+  </si>
+  <si>
+    <t>Field (United Republic of Tanzania_1.0)</t>
+  </si>
+  <si>
+    <t>Field (Zambia_1.0)</t>
+  </si>
+  <si>
+    <t>Field (Malaysia_1.0)</t>
+  </si>
+  <si>
+    <t>Field (Mozambique_1.0)</t>
+  </si>
+  <si>
+    <t>Field (Indonesia_1.0)</t>
   </si>
 </sst>
 </file>
@@ -591,13 +634,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{817AEF70-9A5F-3743-AAC8-23817F8C98EF}">
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -625,11 +668,8 @@
       <c r="I1" t="s">
         <v>42</v>
       </c>
-      <c r="J1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -658,7 +698,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -687,7 +727,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -716,7 +756,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -745,7 +785,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -774,7 +814,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -803,7 +843,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -832,7 +872,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -861,7 +901,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -890,7 +930,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>11</v>
       </c>
@@ -919,7 +959,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>12</v>
       </c>
@@ -927,13 +967,13 @@
         <v>8</v>
       </c>
       <c r="C12">
-        <v>832</v>
+        <v>1183</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12">
-        <v>1200</v>
+        <v>30</v>
+      </c>
+      <c r="E12" t="s">
+        <v>28</v>
       </c>
       <c r="F12" t="s">
         <v>35</v>
@@ -948,7 +988,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>13</v>
       </c>
@@ -977,7 +1017,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>14</v>
       </c>
@@ -1006,7 +1046,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>15</v>
       </c>
@@ -1035,7 +1075,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>16</v>
       </c>
@@ -1390,14 +1430,14 @@
       <c r="B28" t="s">
         <v>23</v>
       </c>
-      <c r="C28" t="s">
-        <v>28</v>
+      <c r="C28">
+        <v>54</v>
       </c>
       <c r="D28" t="s">
-        <v>32</v>
-      </c>
-      <c r="E28">
-        <v>100</v>
+        <v>30</v>
+      </c>
+      <c r="E28" t="s">
+        <v>28</v>
       </c>
       <c r="F28" t="s">
         <v>35</v>
@@ -1448,14 +1488,14 @@
       <c r="B30" t="s">
         <v>24</v>
       </c>
-      <c r="C30" t="s">
-        <v>28</v>
+      <c r="C30">
+        <v>217</v>
       </c>
       <c r="D30" t="s">
-        <v>32</v>
-      </c>
-      <c r="E30">
-        <v>40</v>
+        <v>30</v>
+      </c>
+      <c r="E30" t="s">
+        <v>28</v>
       </c>
       <c r="F30" t="s">
         <v>35</v>
@@ -1477,14 +1517,14 @@
       <c r="B31" t="s">
         <v>25</v>
       </c>
-      <c r="C31" t="s">
-        <v>28</v>
+      <c r="C31">
+        <v>17</v>
       </c>
       <c r="D31" t="s">
         <v>32</v>
       </c>
       <c r="E31">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F31" t="s">
         <v>35</v>
@@ -1997,7 +2037,7 @@
         <v>49</v>
       </c>
       <c r="B49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C49" t="s">
         <v>28</v>
@@ -2026,7 +2066,7 @@
         <v>50</v>
       </c>
       <c r="B50" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C50">
         <v>490</v>
@@ -2047,6 +2087,35 @@
         <v>13.48531966088</v>
       </c>
       <c r="I50" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>51</v>
+      </c>
+      <c r="B51" t="s">
+        <v>68</v>
+      </c>
+      <c r="C51">
+        <v>4</v>
+      </c>
+      <c r="D51" t="s">
+        <v>32</v>
+      </c>
+      <c r="E51">
+        <v>20</v>
+      </c>
+      <c r="F51" t="s">
+        <v>35</v>
+      </c>
+      <c r="G51">
+        <v>43.009601022673898</v>
+      </c>
+      <c r="H51">
+        <v>-81.273722871164296</v>
+      </c>
+      <c r="I51" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2074,7 +2143,7 @@
         <v>29</v>
       </c>
       <c r="D1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E1" t="s">
         <v>38</v>
@@ -2268,7 +2337,7 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C11">
         <v>1183</v>
@@ -3008,7 +3077,7 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C48">
         <v>138</v>
@@ -3028,7 +3097,7 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C49">
         <v>490</v>
@@ -3041,6 +3110,486 @@
       </c>
       <c r="F49" t="s">
         <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2BB37B5-50A5-E14E-8028-BD9D573F05B3}">
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>30</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2">
+        <v>31.6313618324881</v>
+      </c>
+      <c r="H2">
+        <v>120.81527090382799</v>
+      </c>
+      <c r="I2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3">
+        <v>357</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3">
+        <v>13.7472498876686</v>
+      </c>
+      <c r="H3">
+        <v>79.597894056204098</v>
+      </c>
+      <c r="I3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4">
+        <v>1169</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4">
+        <v>9.8771799999999992</v>
+      </c>
+      <c r="H4">
+        <v>8.9792400000000008</v>
+      </c>
+      <c r="I4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5">
+        <v>1.6134820000000001</v>
+      </c>
+      <c r="H5">
+        <v>10.882453</v>
+      </c>
+      <c r="I5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6">
+        <v>184</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6">
+        <v>-16.808704121322599</v>
+      </c>
+      <c r="H6">
+        <v>26.986449529706899</v>
+      </c>
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7">
+        <v>2134</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7">
+        <v>14.3109540738653</v>
+      </c>
+      <c r="H7">
+        <v>101.53044149511599</v>
+      </c>
+      <c r="I7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8">
+        <v>61</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8">
+        <v>4.5984999999999996</v>
+      </c>
+      <c r="H8">
+        <v>101.44019400000001</v>
+      </c>
+      <c r="I8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9">
+        <v>89</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9">
+        <v>0.30488560831545503</v>
+      </c>
+      <c r="H9">
+        <v>34.878761191646099</v>
+      </c>
+      <c r="I9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10">
+        <v>893</v>
+      </c>
+      <c r="D10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10">
+        <v>1.6134820000000001</v>
+      </c>
+      <c r="H10">
+        <v>10.882453</v>
+      </c>
+      <c r="I10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11">
+        <v>121</v>
+      </c>
+      <c r="D11" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11">
+        <v>7.9179002711623898</v>
+      </c>
+      <c r="H11">
+        <v>-1.1574159431062001</v>
+      </c>
+      <c r="I11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12">
+        <v>110</v>
+      </c>
+      <c r="D12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G12">
+        <v>-6.4753175814336696</v>
+      </c>
+      <c r="H12">
+        <v>34.980692564635604</v>
+      </c>
+      <c r="I12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13">
+        <v>51</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13">
+        <v>-16.808704121322599</v>
+      </c>
+      <c r="H13">
+        <v>26.986449529706899</v>
+      </c>
+      <c r="I13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14">
+        <v>20</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14">
+        <v>4.5984999999999996</v>
+      </c>
+      <c r="H14">
+        <v>101.44019400000001</v>
+      </c>
+      <c r="I14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>-18.5865979146634</v>
+      </c>
+      <c r="H15">
+        <v>34.937897765941798</v>
+      </c>
+      <c r="I15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" t="s">
+        <v>36</v>
+      </c>
+      <c r="G16">
+        <v>-7.4326110745669602</v>
+      </c>
+      <c r="H16">
+        <v>111.381131232702</v>
+      </c>
+      <c r="I16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C17">
+        <f>SUM(C2:C9)</f>
+        <v>4077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made a separate file and output for the Sex sensitivity analyses which is distinct from the main model, now re-running main model, outputs will be stored with _main suffix.rds
</commit_message>
<xml_diff>
--- a/data/Holdings/Museum_map.xlsx
+++ b/data/Holdings/Museum_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brinda/Documents/MRes project/data/Holdings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A164480A-D911-5644-A9A0-701D9501C743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B85A5E7A-5931-DE4B-800B-B5000EF193BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1580" yWindow="2000" windowWidth="26440" windowHeight="14280" activeTab="2" xr2:uid="{C4C7C71C-19E0-2247-8E7D-B844CAD8A477}"/>
+    <workbookView xWindow="1580" yWindow="2000" windowWidth="26440" windowHeight="14280" xr2:uid="{C4C7C71C-19E0-2247-8E7D-B844CAD8A477}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="83">
   <si>
     <t>Sr. No</t>
   </si>
@@ -283,6 +283,9 @@
   </si>
   <si>
     <t>Field (Indonesia_1.0)</t>
+  </si>
+  <si>
+    <t>ZFMK1</t>
   </si>
 </sst>
 </file>
@@ -634,10 +637,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{817AEF70-9A5F-3743-AAC8-23817F8C98EF}">
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="54.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -677,7 +680,7 @@
         <v>2</v>
       </c>
       <c r="C2">
-        <v>532</v>
+        <v>689</v>
       </c>
       <c r="D2" t="s">
         <v>30</v>
@@ -764,7 +767,7 @@
         <v>5</v>
       </c>
       <c r="C5">
-        <v>84</v>
+        <v>173</v>
       </c>
       <c r="D5" t="s">
         <v>30</v>
@@ -822,13 +825,13 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <v>24</v>
+        <v>68</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7">
-        <v>100</v>
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>28</v>
       </c>
       <c r="F7" t="s">
         <v>35</v>
@@ -880,7 +883,7 @@
         <v>57</v>
       </c>
       <c r="C9">
-        <v>236</v>
+        <v>278</v>
       </c>
       <c r="D9" t="s">
         <v>30</v>
@@ -967,7 +970,7 @@
         <v>8</v>
       </c>
       <c r="C12">
-        <v>1183</v>
+        <v>1049</v>
       </c>
       <c r="D12" t="s">
         <v>30</v>
@@ -1083,13 +1086,13 @@
         <v>12</v>
       </c>
       <c r="C16">
-        <v>80</v>
+        <v>148</v>
       </c>
       <c r="D16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E16">
-        <v>300</v>
+        <v>30</v>
+      </c>
+      <c r="E16" t="s">
+        <v>28</v>
       </c>
       <c r="F16" t="s">
         <v>35</v>
@@ -1141,7 +1144,7 @@
         <v>14</v>
       </c>
       <c r="C18">
-        <v>501</v>
+        <v>602</v>
       </c>
       <c r="D18" t="s">
         <v>30</v>
@@ -1169,14 +1172,14 @@
       <c r="B19" t="s">
         <v>15</v>
       </c>
-      <c r="C19" t="s">
-        <v>28</v>
+      <c r="C19">
+        <v>39</v>
       </c>
       <c r="D19" t="s">
-        <v>32</v>
-      </c>
-      <c r="E19">
-        <v>50</v>
+        <v>30</v>
+      </c>
+      <c r="E19" t="s">
+        <v>28</v>
       </c>
       <c r="F19" t="s">
         <v>35</v>
@@ -1285,14 +1288,14 @@
       <c r="B23" t="s">
         <v>19</v>
       </c>
-      <c r="C23" t="s">
-        <v>28</v>
+      <c r="C23">
+        <v>266</v>
       </c>
       <c r="D23" t="s">
-        <v>32</v>
-      </c>
-      <c r="E23">
-        <v>300</v>
+        <v>30</v>
+      </c>
+      <c r="E23" t="s">
+        <v>28</v>
       </c>
       <c r="F23" t="s">
         <v>35</v>
@@ -1314,14 +1317,14 @@
       <c r="B24" t="s">
         <v>20</v>
       </c>
-      <c r="C24" t="s">
-        <v>28</v>
+      <c r="C24">
+        <v>46</v>
       </c>
       <c r="D24" t="s">
         <v>32</v>
       </c>
       <c r="E24">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="F24" t="s">
         <v>35</v>
@@ -1466,7 +1469,7 @@
         <v>32</v>
       </c>
       <c r="E29">
-        <v>900</v>
+        <v>500</v>
       </c>
       <c r="F29" t="s">
         <v>35</v>
@@ -1518,13 +1521,13 @@
         <v>25</v>
       </c>
       <c r="C31">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E31">
-        <v>30</v>
+        <v>30</v>
+      </c>
+      <c r="E31" t="s">
+        <v>28</v>
       </c>
       <c r="F31" t="s">
         <v>35</v>
@@ -1546,14 +1549,14 @@
       <c r="B32" t="s">
         <v>26</v>
       </c>
-      <c r="C32" t="s">
-        <v>28</v>
+      <c r="C32">
+        <v>183</v>
       </c>
       <c r="D32" t="s">
-        <v>32</v>
-      </c>
-      <c r="E32">
-        <v>100</v>
+        <v>30</v>
+      </c>
+      <c r="E32" t="s">
+        <v>28</v>
       </c>
       <c r="F32" t="s">
         <v>35</v>
@@ -1979,7 +1982,7 @@
         <v>47</v>
       </c>
       <c r="B47" t="s">
-        <v>54</v>
+        <v>82</v>
       </c>
       <c r="C47">
         <v>83</v>
@@ -2116,6 +2119,35 @@
         <v>-81.273722871164296</v>
       </c>
       <c r="I51" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>52</v>
+      </c>
+      <c r="B52" t="s">
+        <v>54</v>
+      </c>
+      <c r="C52">
+        <v>73</v>
+      </c>
+      <c r="D52" t="s">
+        <v>30</v>
+      </c>
+      <c r="E52" t="s">
+        <v>28</v>
+      </c>
+      <c r="F52" t="s">
+        <v>35</v>
+      </c>
+      <c r="G52">
+        <v>50.722367246940202</v>
+      </c>
+      <c r="H52">
+        <v>7.1135518254663301</v>
+      </c>
+      <c r="I52" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update analysis files and remove sensitive data
</commit_message>
<xml_diff>
--- a/data/Holdings/Museum_map.xlsx
+++ b/data/Holdings/Museum_map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brinda/Documents/MRes project/data/Holdings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B85A5E7A-5931-DE4B-800B-B5000EF193BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A60C8A-6AC2-9F47-8DFB-0F81E1BEF0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1580" yWindow="2000" windowWidth="26440" windowHeight="14280" xr2:uid="{C4C7C71C-19E0-2247-8E7D-B844CAD8A477}"/>
   </bookViews>
@@ -1666,7 +1666,7 @@
         <v>45</v>
       </c>
       <c r="C36">
-        <v>1000</v>
+        <v>1636</v>
       </c>
       <c r="D36" t="s">
         <v>30</v>

</xml_diff>